<commit_message>
Add Seventh Batch cleaned datasets
</commit_message>
<xml_diff>
--- a/data/cleaned/cleaned_swq_manual_physical_parameters_cpcb_ar_2021_2025.xlsx
+++ b/data/cleaned/cleaned_swq_manual_physical_parameters_cpcb_ar_2021_2025.xlsx
@@ -626,7 +626,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>06-01-2021 08:30</t>
+          <t>2021-06-01 08:30:00</t>
         </is>
       </c>
       <c r="T2" t="inlineStr"/>
@@ -719,7 +719,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>08-02-2021 08:30</t>
+          <t>2021-08-02 08:30:00</t>
         </is>
       </c>
       <c r="T3" t="inlineStr"/>
@@ -812,7 +812,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>02-03-2021 08:30</t>
+          <t>2021-02-03 08:30:00</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>

</xml_diff>